<commit_message>
Re-doing script for writing psutlr.xlsx file
</commit_message>
<xml_diff>
--- a/data/psutlr.xlsx
+++ b/data/psutlr.xlsx
@@ -6,44 +6,44 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Transport_E_Final_1900" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transport_E_Useful_1900" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="world_electricity_X_Final_1900" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="world_electricity_X_Useful_1900" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="R__Transport_E_Final_1900">'Transport_E_Final_1900'!$A$78:$Q$82</definedName>
-    <definedName name="U__Transport_E_Final_1900">'Transport_E_Final_1900'!$T$41:$AG$57</definedName>
-    <definedName name="V__Transport_E_Final_1900">'Transport_E_Final_1900'!$A$61:$Q$74</definedName>
-    <definedName name="Y__Transport_E_Final_1900">'Transport_E_Final_1900'!$AJ$41:$AN$57</definedName>
-    <definedName name="r_EIOU__Transport_E_Final_1900">'Transport_E_Final_1900'!$AJ$1:$AW$17</definedName>
-    <definedName name="U_EIOU__Transport_E_Final_1900">'Transport_E_Final_1900'!$T$1:$AG$17</definedName>
-    <definedName name="U_feed__Transport_E_Final_1900">'Transport_E_Final_1900'!$T$21:$AG$37</definedName>
-    <definedName name="S_units__Transport_E_Final_1900">'Transport_E_Final_1900'!$A$1:$B$22</definedName>
-    <definedName name="R__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$A$98:$V$102</definedName>
-    <definedName name="U__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$Y$51:$AQ$72</definedName>
-    <definedName name="V__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$A$76:$V$94</definedName>
-    <definedName name="Y__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$AT$51:$AV$72</definedName>
-    <definedName name="r_EIOU__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$AT$1:$BL$22</definedName>
-    <definedName name="U_EIOU__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$Y$1:$AQ$22</definedName>
-    <definedName name="U_feed__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$Y$26:$AQ$47</definedName>
-    <definedName name="S_units__Transport_E_Useful_1900">'Transport_E_Useful_1900'!$A$1:$B$22</definedName>
-    <definedName name="R__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$A$40:$G$42</definedName>
-    <definedName name="U__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$J$21:$O$27</definedName>
-    <definedName name="V__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$A$31:$G$36</definedName>
-    <definedName name="Y__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$R$21:$Y$27</definedName>
-    <definedName name="r_EIOU__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$R$1:$W$7</definedName>
-    <definedName name="U_EIOU__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$J$1:$O$7</definedName>
-    <definedName name="U_feed__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$J$11:$O$17</definedName>
-    <definedName name="S_units__world_electricity_X_Final_1900">'world_electricity_X_Final_1900'!$A$1:$B$16</definedName>
-    <definedName name="R__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$A$76:$P$78</definedName>
-    <definedName name="U__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$S$39:$AG$54</definedName>
-    <definedName name="V__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$A$58:$P$72</definedName>
-    <definedName name="Y__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$AJ$39:$AQ$54</definedName>
-    <definedName name="r_EIOU__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$AJ$1:$AX$16</definedName>
-    <definedName name="U_EIOU__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$S$1:$AG$16</definedName>
-    <definedName name="U_feed__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$S$20:$AG$35</definedName>
-    <definedName name="S_units__world_electricity_X_Useful_1900">'world_electricity_X_Useful_1900'!$A$1:$B$16</definedName>
+    <definedName name="R__1">'1'!$A$78:$Q$82</definedName>
+    <definedName name="U__1">'1'!$T$41:$AG$57</definedName>
+    <definedName name="V__1">'1'!$A$61:$Q$74</definedName>
+    <definedName name="Y__1">'1'!$AJ$41:$AN$57</definedName>
+    <definedName name="r_EIOU__1">'1'!$AJ$1:$AW$17</definedName>
+    <definedName name="U_EIOU__1">'1'!$T$1:$AG$17</definedName>
+    <definedName name="U_feed__1">'1'!$T$21:$AG$37</definedName>
+    <definedName name="S_units__1">'1'!$A$1:$B$22</definedName>
+    <definedName name="R__2">'2'!$A$98:$V$102</definedName>
+    <definedName name="U__2">'2'!$Y$51:$AQ$72</definedName>
+    <definedName name="V__2">'2'!$A$76:$V$94</definedName>
+    <definedName name="Y__2">'2'!$AT$51:$AV$72</definedName>
+    <definedName name="r_EIOU__2">'2'!$AT$1:$BL$22</definedName>
+    <definedName name="U_EIOU__2">'2'!$Y$1:$AQ$22</definedName>
+    <definedName name="U_feed__2">'2'!$Y$26:$AQ$47</definedName>
+    <definedName name="S_units__2">'2'!$A$1:$B$22</definedName>
+    <definedName name="R__3">'3'!$A$40:$G$42</definedName>
+    <definedName name="U__3">'3'!$J$21:$O$27</definedName>
+    <definedName name="V__3">'3'!$A$31:$G$36</definedName>
+    <definedName name="Y__3">'3'!$R$21:$Y$27</definedName>
+    <definedName name="r_EIOU__3">'3'!$R$1:$W$7</definedName>
+    <definedName name="U_EIOU__3">'3'!$J$1:$O$7</definedName>
+    <definedName name="U_feed__3">'3'!$J$11:$O$17</definedName>
+    <definedName name="S_units__3">'3'!$A$1:$B$16</definedName>
+    <definedName name="R__4">'4'!$A$76:$P$78</definedName>
+    <definedName name="U__4">'4'!$S$39:$AG$54</definedName>
+    <definedName name="V__4">'4'!$A$58:$P$72</definedName>
+    <definedName name="Y__4">'4'!$AJ$39:$AQ$54</definedName>
+    <definedName name="r_EIOU__4">'4'!$AJ$1:$AX$16</definedName>
+    <definedName name="U_EIOU__4">'4'!$S$1:$AG$16</definedName>
+    <definedName name="U_feed__4">'4'!$S$20:$AG$35</definedName>
+    <definedName name="S_units__4">'4'!$A$1:$B$16</definedName>
   </definedNames>
 </workbook>
 </file>

</xml_diff>

<commit_message>
Updated files from Ricardo.
</commit_message>
<xml_diff>
--- a/data/psutlr.xlsx
+++ b/data/psutlr.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Transport_E_Final_2017" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="world_electricity_X_Final_2017" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="WorldElectricity_X_Final_2017" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="R__Transport_E_Final_2017">'Transport_E_Final_2017'!$A$202:$AY$217</definedName>
@@ -18,40 +18,40 @@
     <definedName name="U_EIOU__Transport_E_Final_2017">'Transport_E_Final_2017'!$BB$1:$CK$51</definedName>
     <definedName name="U_feed__Transport_E_Final_2017">'Transport_E_Final_2017'!$BB$55:$CK$105</definedName>
     <definedName name="S_units__Transport_E_Final_2017">'Transport_E_Final_2017'!$A$1:$B$63</definedName>
-    <definedName name="R__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$A$133:$AE$147</definedName>
-    <definedName name="U__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$AH$69:$BH$99</definedName>
-    <definedName name="V__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$A$103:$AE$129</definedName>
-    <definedName name="Y__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$BK$69:$BS$99</definedName>
-    <definedName name="r_EIOU__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$BK$1:$CK$31</definedName>
-    <definedName name="U_EIOU__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$AH$1:$BH$31</definedName>
-    <definedName name="U_feed__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$AH$35:$BH$65</definedName>
-    <definedName name="S_units__world_electricity_X_Final_2017">'world_electricity_X_Final_2017'!$A$1:$B$44</definedName>
+    <definedName name="R__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$A$133:$AE$147</definedName>
+    <definedName name="U__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$AH$69:$BH$99</definedName>
+    <definedName name="V__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$A$103:$AE$129</definedName>
+    <definedName name="Y__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$BK$69:$BS$99</definedName>
+    <definedName name="r_EIOU__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$BK$1:$CK$31</definedName>
+    <definedName name="U_EIOU__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$AH$1:$BH$31</definedName>
+    <definedName name="U_feed__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$AH$35:$BH$65</definedName>
+    <definedName name="S_units__WorldElectricity_X_Final_2017">'WorldElectricity_X_Final_2017'!$A$1:$B$44</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">Aviation Gasoline [from Oil Pipeline]</t>
+    <t xml:space="preserve">Aviation gasoline</t>
   </si>
   <si>
-    <t xml:space="preserve">Aviation Gasoline [from Oil Refinery]</t>
+    <t xml:space="preserve">Aviation gasoline [from Oil refineries]</t>
   </si>
   <si>
-    <t xml:space="preserve">Coal and coal products (if no detail) [from Coal mines]</t>
+    <t xml:space="preserve">Coal &amp; coal products</t>
   </si>
   <si>
-    <t xml:space="preserve">Coal and coal products (if no detail) [from Resources]</t>
+    <t xml:space="preserve">Coal &amp; coal products (if no detail) [from Coal mines]</t>
   </si>
   <si>
-    <t xml:space="preserve">Coal And Coal Products [from Coal depot]</t>
+    <t xml:space="preserve">Coal &amp; coal products (if no detail) [from Resources]</t>
   </si>
   <si>
-    <t xml:space="preserve">Coal And Coal Products [from Coal distribution]</t>
+    <t xml:space="preserve">Coal &amp; coal Products [from Coal depot]</t>
   </si>
   <si>
     <t xml:space="preserve">Combustible renewables [from Manufacture]</t>
@@ -60,10 +60,7 @@
     <t xml:space="preserve">Combustible renewables [from Resources]</t>
   </si>
   <si>
-    <t xml:space="preserve">Diesel [from Oil Pipeline]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diesel [from Oil Refinery]</t>
+    <t xml:space="preserve">Diesel [from Oil refineries]</t>
   </si>
   <si>
     <t xml:space="preserve">Electricity</t>
@@ -72,16 +69,16 @@
     <t xml:space="preserve">Electricity (Pre-Distribution)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuel Oil [from Oil Pipeline]</t>
+    <t xml:space="preserve">Fuel oil</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuel Oil [from Oil Refinery]</t>
+    <t xml:space="preserve">Fuel oil [from Oil refineries]</t>
   </si>
   <si>
-    <t xml:space="preserve">Gasoline [from Oil Pipeline]</t>
+    <t xml:space="preserve">Gas/diesel oil excl. biofuels</t>
   </si>
   <si>
-    <t xml:space="preserve">Gasoline [from Oil Refinery]</t>
+    <t xml:space="preserve">Gasoline [from Oil refineries]</t>
   </si>
   <si>
     <t xml:space="preserve">Geothermal [from Manufacture]</t>
@@ -96,25 +93,25 @@
     <t xml:space="preserve">Hydro [from Resources]</t>
   </si>
   <si>
-    <t xml:space="preserve">Jet Fuel [from Oil Pipeline]</t>
+    <t xml:space="preserve">Jet fuel</t>
   </si>
   <si>
-    <t xml:space="preserve">Jet Fuel [from Oil Refinery]</t>
+    <t xml:space="preserve">Jet fuel [from Oil refineries]</t>
   </si>
   <si>
-    <t xml:space="preserve">Liquid Biofuels [from Biofuel Pipeline]</t>
+    <t xml:space="preserve">Liquid biofuels [from Biofuel refineries]</t>
   </si>
   <si>
-    <t xml:space="preserve">Liquid Biofuels [from Biofuel Refinery]</t>
+    <t xml:space="preserve">Motor gasoline excl. biofuels</t>
   </si>
   <si>
-    <t xml:space="preserve">Natural Gas [from Natural gas extraction]</t>
+    <t xml:space="preserve">Natural gas</t>
   </si>
   <si>
-    <t xml:space="preserve">Natural Gas [from Natural Gas Pipeline]</t>
+    <t xml:space="preserve">Natural gas [from Natural gas extraction]</t>
   </si>
   <si>
-    <t xml:space="preserve">Natural Gas [from Natural Gas storage]</t>
+    <t xml:space="preserve">Natural gas [from Natural gas storage]</t>
   </si>
   <si>
     <t xml:space="preserve">Natural Gas [from Resources]</t>
@@ -132,10 +129,10 @@
     <t xml:space="preserve">Nuclear [from Resources]</t>
   </si>
   <si>
-    <t xml:space="preserve">Oil and oil products (if no detail) [from Oil extraction]</t>
+    <t xml:space="preserve">Oil &amp; oil products (if no detail) [from Oil extraction]</t>
   </si>
   <si>
-    <t xml:space="preserve">Oil and oil products (if no detail) [from Resources]</t>
+    <t xml:space="preserve">Oil &amp; oil products (if no detail) [from Resources]</t>
   </si>
   <si>
     <t xml:space="preserve">Other [from Manufacture]</t>
@@ -144,10 +141,13 @@
     <t xml:space="preserve">Other [from Resources]</t>
   </si>
   <si>
-    <t xml:space="preserve">Other Petroleum Products [from Oil Pipeline]</t>
+    <t xml:space="preserve">Other liquid biofuels</t>
   </si>
   <si>
-    <t xml:space="preserve">Other Petroleum Products [from Oil Refinery]</t>
+    <t xml:space="preserve">Other petroleum products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other petroleum products [from Oil refineries]</t>
   </si>
   <si>
     <t xml:space="preserve">Peat [from Manufacture]</t>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">Wind [from Resources]</t>
   </si>
   <si>
-    <t xml:space="preserve">Resources [of Coal and coal products (if no detail)]</t>
+    <t xml:space="preserve">Resources [of Coal &amp; coal products (if no detail)]</t>
   </si>
   <si>
     <t xml:space="preserve">Resources [of Combustible renewables]</t>
@@ -207,7 +207,7 @@
     <t xml:space="preserve">Resources [of Nuclear]</t>
   </si>
   <si>
-    <t xml:space="preserve">Resources [of Oil and oil products (if no detail)]</t>
+    <t xml:space="preserve">Resources [of Oil &amp; oil products (if no detail)]</t>
   </si>
   <si>
     <t xml:space="preserve">Resources [of Other]</t>
@@ -234,13 +234,13 @@
     <t xml:space="preserve">R</t>
   </si>
   <si>
-    <t xml:space="preserve">Biofuel Pipeline</t>
+    <t xml:space="preserve">Biofuel pipelines</t>
   </si>
   <si>
-    <t xml:space="preserve">Biofuel Refinery</t>
+    <t xml:space="preserve">Biofuel refineries</t>
   </si>
   <si>
-    <t xml:space="preserve">Biomass Powerplant</t>
+    <t xml:space="preserve">Biomass powerplants</t>
   </si>
   <si>
     <t xml:space="preserve">Coal depot</t>
@@ -249,19 +249,19 @@
     <t xml:space="preserve">Coal distribution</t>
   </si>
   <si>
-    <t xml:space="preserve">Coal Mines</t>
+    <t xml:space="preserve">Coal mines</t>
   </si>
   <si>
-    <t xml:space="preserve">Coal Powerplant</t>
+    <t xml:space="preserve">Coal powerplants</t>
   </si>
   <si>
-    <t xml:space="preserve">Geothermal Powerplant</t>
+    <t xml:space="preserve">Geothermal powerplants</t>
   </si>
   <si>
-    <t xml:space="preserve">Grid Transportation</t>
+    <t xml:space="preserve">Grid transportation</t>
   </si>
   <si>
-    <t xml:space="preserve">Hydro Powerplant</t>
+    <t xml:space="preserve">Hydro powerplants</t>
   </si>
   <si>
     <t xml:space="preserve">Manufacture [of Combustible renewables]</t>
@@ -303,40 +303,40 @@
     <t xml:space="preserve">Natural gas extraction</t>
   </si>
   <si>
-    <t xml:space="preserve">Natural Gas Pipeline</t>
+    <t xml:space="preserve">Natural gas pipelines</t>
   </si>
   <si>
-    <t xml:space="preserve">Natural Gas Powerplant</t>
+    <t xml:space="preserve">Natural gas powerplants</t>
   </si>
   <si>
-    <t xml:space="preserve">Natural Gas storage</t>
+    <t xml:space="preserve">Natural gas storage</t>
   </si>
   <si>
-    <t xml:space="preserve">Nuclear Powerplant</t>
+    <t xml:space="preserve">Nuclear powerplants</t>
   </si>
   <si>
     <t xml:space="preserve">Oil extraction</t>
   </si>
   <si>
-    <t xml:space="preserve">Oil Pipeline</t>
+    <t xml:space="preserve">Oil pipelines</t>
   </si>
   <si>
-    <t xml:space="preserve">Oil Powerplant</t>
+    <t xml:space="preserve">Oil powerplants</t>
   </si>
   <si>
-    <t xml:space="preserve">Oil Refinery</t>
+    <t xml:space="preserve">Oil refineries</t>
   </si>
   <si>
-    <t xml:space="preserve">Solar Pv Panel</t>
+    <t xml:space="preserve">Solar photovoltaic panels</t>
   </si>
   <si>
-    <t xml:space="preserve">Solar Thermal Panel</t>
+    <t xml:space="preserve">Solar thermal panels</t>
   </si>
   <si>
-    <t xml:space="preserve">Wave Turbine</t>
+    <t xml:space="preserve">Wave turbines</t>
   </si>
   <si>
-    <t xml:space="preserve">Wind Turbine</t>
+    <t xml:space="preserve">Wind turbines</t>
   </si>
   <si>
     <t xml:space="preserve">U</t>
@@ -372,112 +372,49 @@
     <t xml:space="preserve">TJ</t>
   </si>
   <si>
-    <t xml:space="preserve">AirP [from Jet Aircrafts]</t>
+    <t xml:space="preserve">AirP [from Jet aircrafts]</t>
   </si>
   <si>
-    <t xml:space="preserve">AirP [from Piston Aircrafts]</t>
+    <t xml:space="preserve">AirP [from Piston aircrafts]</t>
   </si>
   <si>
-    <t xml:space="preserve">MaP [from Coal Steam Ships]</t>
+    <t xml:space="preserve">MaP [from Coal steam ships]</t>
   </si>
   <si>
-    <t xml:space="preserve">MaP [from Oil Ships]</t>
+    <t xml:space="preserve">MaP [from Oil ships]</t>
   </si>
   <si>
-    <t xml:space="preserve">RaP [from Diesel Trains]</t>
+    <t xml:space="preserve">RaP [from Diesel trains]</t>
   </si>
   <si>
-    <t xml:space="preserve">RaP [from Electric Trains]</t>
+    <t xml:space="preserve">RaP [from Electric trains]</t>
   </si>
   <si>
-    <t xml:space="preserve">RaP [from Steam Trains]</t>
+    <t xml:space="preserve">RaP [from Steam trains]</t>
   </si>
   <si>
-    <t xml:space="preserve">RoP [from Diesel Vehicles]</t>
+    <t xml:space="preserve">RoP [from Diesel vehicles]</t>
   </si>
   <si>
-    <t xml:space="preserve">RoP [from Electric Vehicles]</t>
+    <t xml:space="preserve">RoP [from Electric vehicles]</t>
   </si>
   <si>
-    <t xml:space="preserve">RoP [from Gasoline Or Diesel Vehicles]</t>
+    <t xml:space="preserve">RoP [from gasoline or diesel vehicles]</t>
   </si>
   <si>
-    <t xml:space="preserve">RoP [from Gasoline Vehicles]</t>
+    <t xml:space="preserve">RoP [from Gasoline vehicles]</t>
   </si>
   <si>
-    <t xml:space="preserve">RoP [from Natural Gas Vehicles]</t>
+    <t xml:space="preserve">RoP [from Natural gas vehicles]</t>
   </si>
   <si>
     <t xml:space="preserve">S_units</t>
   </si>
   <si>
-    <t xml:space="preserve">Combustible renewables [from Manufacture [of Combustible renewables]]</t>
-  </si>
-  <si>
     <t xml:space="preserve">Electricity (pre-distribution)</t>
   </si>
   <si>
-    <t xml:space="preserve">Geothermal [from Manufacture [of Geothermal]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hydro [from Manufacture [of Hydro]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuclear [from Manufacture [of Nuclear]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other [from Manufacture [of Other]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peat [from Manufacture [of Peat]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solar photovoltaics [from Manufacture [of Solar photovoltaics]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solar thermal [from Manufacture [of Solar thermal]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tide, wave and ocean [from Manufacture [of Tide, wave, and ocean]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waste (if no detail) [from Manufacture [of Waste (if no detail)]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wind [from Manufacture [of Wind]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biomass powerplants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coal mines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coal powerplants</t>
-  </si>
-  <si>
     <t xml:space="preserve">Electricity grid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geothermal powerplants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hydro powerplants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Natural gas powerplants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuclear powerplants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oil powerplants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solar PV panels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solar thermal panels</t>
   </si>
   <si>
     <t xml:space="preserve">Unspecified</t>
@@ -541,9 +478,6 @@
   </si>
   <si>
     <t xml:space="preserve">MTH.100.C [from Electric stoves]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RaP [from Electric trains]</t>
   </si>
 </sst>
 </file>
@@ -6643,10 +6577,10 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>23</v>
+        <v>115</v>
       </c>
       <c r="B26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BB26" s="4" t="s">
         <v>25</v>
@@ -6867,10 +6801,10 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="B27" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BB27" s="4" t="s">
         <v>26</v>
@@ -7091,10 +7025,10 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="s">
-        <v>115</v>
+        <v>23</v>
       </c>
       <c r="B28" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB28" s="4" t="s">
         <v>27</v>
@@ -7315,10 +7249,10 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="B29" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB29" s="4" t="s">
         <v>28</v>
@@ -12865,7 +12799,7 @@
         <v>0</v>
       </c>
       <c r="BF58" s="7" t="n">
-        <v>5353.1838648</v>
+        <v>0</v>
       </c>
       <c r="BG58" s="7" t="n">
         <v>0</v>
@@ -12874,7 +12808,7 @@
         <v>0</v>
       </c>
       <c r="BI58" s="7" t="n">
-        <v>1225536.11315653</v>
+        <v>0</v>
       </c>
       <c r="BJ58" s="7" t="n">
         <v>0</v>
@@ -12981,16 +12915,16 @@
         <v>0</v>
       </c>
       <c r="BF59" s="7" t="n">
-        <v>0</v>
+        <v>5353.1838648</v>
       </c>
       <c r="BG59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="BH59" s="7" t="n">
-        <v>1230889.29702133</v>
+        <v>0</v>
       </c>
       <c r="BI59" s="7" t="n">
-        <v>0</v>
+        <v>1225536.11315653</v>
       </c>
       <c r="BJ59" s="7" t="n">
         <v>0</v>
@@ -13100,10 +13034,10 @@
         <v>0</v>
       </c>
       <c r="BG60" s="7" t="n">
-        <v>5353.1838648</v>
+        <v>0</v>
       </c>
       <c r="BH60" s="7" t="n">
-        <v>0</v>
+        <v>1230889.29702133</v>
       </c>
       <c r="BI60" s="7" t="n">
         <v>0</v>
@@ -13216,7 +13150,7 @@
         <v>0</v>
       </c>
       <c r="BG61" s="7" t="n">
-        <v>0</v>
+        <v>5353.1838648</v>
       </c>
       <c r="BH61" s="7" t="n">
         <v>0</v>
@@ -13634,7 +13568,7 @@
         <v>0</v>
       </c>
       <c r="CE64" s="7" t="n">
-        <v>0</v>
+        <v>40635892.6447752</v>
       </c>
       <c r="CF64" s="7" t="n">
         <v>0</v>
@@ -13744,7 +13678,7 @@
         <v>0</v>
       </c>
       <c r="CE65" s="7" t="n">
-        <v>40635892.6447752</v>
+        <v>0</v>
       </c>
       <c r="CF65" s="7" t="n">
         <v>0</v>
@@ -13794,7 +13728,7 @@
         <v>0</v>
       </c>
       <c r="BK66" s="7" t="n">
-        <v>0</v>
+        <v>1253490.86467101</v>
       </c>
       <c r="BL66" s="7" t="n">
         <v>0</v>
@@ -13904,7 +13838,7 @@
         <v>0</v>
       </c>
       <c r="BK67" s="7" t="n">
-        <v>1253490.86467101</v>
+        <v>0</v>
       </c>
       <c r="BL67" s="7" t="n">
         <v>0</v>
@@ -14074,7 +14008,7 @@
         <v>0</v>
       </c>
       <c r="CE68" s="7" t="n">
-        <v>0</v>
+        <v>8005505.001336</v>
       </c>
       <c r="CF68" s="7" t="n">
         <v>0</v>
@@ -14184,7 +14118,7 @@
         <v>0</v>
       </c>
       <c r="CE69" s="7" t="n">
-        <v>8005505.001336</v>
+        <v>0</v>
       </c>
       <c r="CF69" s="7" t="n">
         <v>0</v>
@@ -14294,7 +14228,7 @@
         <v>0</v>
       </c>
       <c r="CE70" s="7" t="n">
-        <v>0</v>
+        <v>45225402.66558</v>
       </c>
       <c r="CF70" s="7" t="n">
         <v>0</v>
@@ -14341,7 +14275,7 @@
         <v>0</v>
       </c>
       <c r="BJ71" s="7" t="n">
-        <v>0</v>
+        <v>27853.346068534</v>
       </c>
       <c r="BK71" s="7" t="n">
         <v>0</v>
@@ -14404,7 +14338,7 @@
         <v>0</v>
       </c>
       <c r="CE71" s="7" t="n">
-        <v>45225402.66558</v>
+        <v>0</v>
       </c>
       <c r="CF71" s="7" t="n">
         <v>0</v>
@@ -14451,19 +14385,19 @@
         <v>0</v>
       </c>
       <c r="BJ72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN72" s="7" t="n">
         <v>27853.346068534</v>
-      </c>
-      <c r="BK72" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL72" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM72" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN72" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="BO72" s="7" t="n">
         <v>0</v>
@@ -14567,13 +14501,13 @@
         <v>0</v>
       </c>
       <c r="BL73" s="7" t="n">
-        <v>0</v>
+        <v>199847.318978253</v>
       </c>
       <c r="BM73" s="7" t="n">
         <v>0</v>
       </c>
       <c r="BN73" s="7" t="n">
-        <v>27853.346068534</v>
+        <v>0</v>
       </c>
       <c r="BO73" s="7" t="n">
         <v>0</v>
@@ -14677,16 +14611,16 @@
         <v>0</v>
       </c>
       <c r="BL74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO74" s="7" t="n">
         <v>199847.318978253</v>
-      </c>
-      <c r="BM74" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN74" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO74" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="BP74" s="7" t="n">
         <v>0</v>
@@ -14796,7 +14730,7 @@
         <v>0</v>
       </c>
       <c r="BO75" s="7" t="n">
-        <v>199847.318978253</v>
+        <v>0</v>
       </c>
       <c r="BP75" s="7" t="n">
         <v>0</v>
@@ -14954,7 +14888,7 @@
         <v>0</v>
       </c>
       <c r="CE76" s="7" t="n">
-        <v>0</v>
+        <v>13528049.1087492</v>
       </c>
       <c r="CF76" s="7" t="n">
         <v>0</v>
@@ -14980,7 +14914,7 @@
         <v>22</v>
       </c>
       <c r="BC77" s="7" t="n">
-        <v>0</v>
+        <v>3347317.4724324</v>
       </c>
       <c r="BD77" s="7" t="n">
         <v>0</v>
@@ -15064,7 +14998,7 @@
         <v>0</v>
       </c>
       <c r="CE77" s="7" t="n">
-        <v>13528049.1087492</v>
+        <v>0</v>
       </c>
       <c r="CF77" s="7" t="n">
         <v>0</v>
@@ -15200,7 +15134,7 @@
         <v>24</v>
       </c>
       <c r="BC79" s="7" t="n">
-        <v>3347317.4724324</v>
+        <v>0</v>
       </c>
       <c r="BD79" s="7" t="n">
         <v>0</v>
@@ -15489,7 +15423,7 @@
         <v>0</v>
       </c>
       <c r="BZ81" s="7" t="n">
-        <v>0</v>
+        <v>1891512.504</v>
       </c>
       <c r="CA81" s="7" t="n">
         <v>0</v>
@@ -15596,10 +15530,10 @@
         <v>0</v>
       </c>
       <c r="BY82" s="7" t="n">
-        <v>0</v>
+        <v>2521699.4809766</v>
       </c>
       <c r="BZ82" s="7" t="n">
-        <v>1891512.504</v>
+        <v>0</v>
       </c>
       <c r="CA82" s="7" t="n">
         <v>0</v>
@@ -15643,7 +15577,7 @@
         <v>0</v>
       </c>
       <c r="BD83" s="7" t="n">
-        <v>0</v>
+        <v>14862828.8108352</v>
       </c>
       <c r="BE83" s="7" t="n">
         <v>0</v>
@@ -15706,7 +15640,7 @@
         <v>0</v>
       </c>
       <c r="BY83" s="7" t="n">
-        <v>2521699.4809766</v>
+        <v>0</v>
       </c>
       <c r="BZ83" s="7" t="n">
         <v>0</v>
@@ -15753,43 +15687,43 @@
         <v>0</v>
       </c>
       <c r="BD84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP84" s="7" t="n">
         <v>14862828.8108352</v>
-      </c>
-      <c r="BE84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP84" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="BQ84" s="7" t="n">
         <v>0</v>
@@ -15899,7 +15833,7 @@
         <v>0</v>
       </c>
       <c r="BP85" s="7" t="n">
-        <v>14862828.8108352</v>
+        <v>0</v>
       </c>
       <c r="BQ85" s="7" t="n">
         <v>0</v>
@@ -15938,7 +15872,7 @@
         <v>0</v>
       </c>
       <c r="CC85" s="7" t="n">
-        <v>0</v>
+        <v>391031.372077766</v>
       </c>
       <c r="CD85" s="7" t="n">
         <v>0</v>
@@ -16012,7 +15946,7 @@
         <v>0</v>
       </c>
       <c r="BQ86" s="7" t="n">
-        <v>0</v>
+        <v>391031.372077766</v>
       </c>
       <c r="BR86" s="7" t="n">
         <v>0</v>
@@ -16048,7 +15982,7 @@
         <v>0</v>
       </c>
       <c r="CC86" s="7" t="n">
-        <v>391031.372077766</v>
+        <v>0</v>
       </c>
       <c r="CD86" s="7" t="n">
         <v>0</v>
@@ -16122,7 +16056,7 @@
         <v>0</v>
       </c>
       <c r="BQ87" s="7" t="n">
-        <v>391031.372077766</v>
+        <v>0</v>
       </c>
       <c r="BR87" s="7" t="n">
         <v>0</v>
@@ -16167,10 +16101,10 @@
         <v>0</v>
       </c>
       <c r="CF87" s="7" t="n">
-        <v>0</v>
+        <v>121834.370880332</v>
       </c>
       <c r="CG87" s="7" t="n">
-        <v>0</v>
+        <v>108477908.839307</v>
       </c>
       <c r="CH87" s="7" t="n">
         <v>0</v>
@@ -16271,16 +16205,16 @@
         <v>0</v>
       </c>
       <c r="CD88" s="7" t="n">
-        <v>0</v>
+        <v>108599743.210187</v>
       </c>
       <c r="CE88" s="7" t="n">
         <v>0</v>
       </c>
       <c r="CF88" s="7" t="n">
-        <v>121834.370880332</v>
+        <v>0</v>
       </c>
       <c r="CG88" s="7" t="n">
-        <v>108477908.839307</v>
+        <v>0</v>
       </c>
       <c r="CH88" s="7" t="n">
         <v>0</v>
@@ -16381,7 +16315,7 @@
         <v>0</v>
       </c>
       <c r="CD89" s="7" t="n">
-        <v>108599743.210187</v>
+        <v>0</v>
       </c>
       <c r="CE89" s="7" t="n">
         <v>0</v>
@@ -16399,7 +16333,7 @@
         <v>0</v>
       </c>
       <c r="CJ89" s="7" t="n">
-        <v>0</v>
+        <v>1763.36022332228</v>
       </c>
       <c r="CK89" s="7" t="n">
         <v>0</v>
@@ -16455,7 +16389,7 @@
         <v>0</v>
       </c>
       <c r="BR90" s="7" t="n">
-        <v>0</v>
+        <v>1763.36022332228</v>
       </c>
       <c r="BS90" s="7" t="n">
         <v>0</v>
@@ -16509,7 +16443,7 @@
         <v>0</v>
       </c>
       <c r="CJ90" s="7" t="n">
-        <v>1763.36022332228</v>
+        <v>0</v>
       </c>
       <c r="CK90" s="7" t="n">
         <v>0</v>
@@ -16565,7 +16499,7 @@
         <v>0</v>
       </c>
       <c r="BR91" s="7" t="n">
-        <v>1763.36022332228</v>
+        <v>0</v>
       </c>
       <c r="BS91" s="7" t="n">
         <v>0</v>
@@ -18560,7 +18494,7 @@
         <v>0</v>
       </c>
       <c r="BF112" s="6" t="n">
-        <v>5353.1838648</v>
+        <v>0</v>
       </c>
       <c r="BG112" s="6" t="n">
         <v>0</v>
@@ -18569,7 +18503,7 @@
         <v>0</v>
       </c>
       <c r="BI112" s="6" t="n">
-        <v>1225536.11315653</v>
+        <v>0</v>
       </c>
       <c r="BJ112" s="6" t="n">
         <v>0</v>
@@ -18662,7 +18596,7 @@
         <v>0</v>
       </c>
       <c r="CP112" s="1" t="n">
-        <v>0</v>
+        <v>5353.1838648</v>
       </c>
       <c r="CQ112" s="1" t="n">
         <v>0</v>
@@ -18685,16 +18619,16 @@
         <v>0</v>
       </c>
       <c r="BF113" s="6" t="n">
-        <v>0</v>
+        <v>5353.1838648</v>
       </c>
       <c r="BG113" s="6" t="n">
         <v>0</v>
       </c>
       <c r="BH113" s="6" t="n">
-        <v>1230889.29702133</v>
+        <v>0</v>
       </c>
       <c r="BI113" s="6" t="n">
-        <v>0</v>
+        <v>1225536.11315653</v>
       </c>
       <c r="BJ113" s="6" t="n">
         <v>0</v>
@@ -18813,10 +18747,10 @@
         <v>0</v>
       </c>
       <c r="BG114" s="6" t="n">
-        <v>5353.1838648</v>
+        <v>0</v>
       </c>
       <c r="BH114" s="6" t="n">
-        <v>0</v>
+        <v>1230889.29702133</v>
       </c>
       <c r="BI114" s="6" t="n">
         <v>0</v>
@@ -18938,7 +18872,7 @@
         <v>0</v>
       </c>
       <c r="BG115" s="6" t="n">
-        <v>0</v>
+        <v>5353.1838648</v>
       </c>
       <c r="BH115" s="6" t="n">
         <v>0</v>
@@ -19037,7 +18971,7 @@
         <v>0</v>
       </c>
       <c r="CP115" s="1" t="n">
-        <v>5353.1838648</v>
+        <v>0</v>
       </c>
       <c r="CQ115" s="1" t="n">
         <v>0</v>
@@ -19385,7 +19319,7 @@
         <v>0</v>
       </c>
       <c r="CE118" s="6" t="n">
-        <v>0</v>
+        <v>40635892.6447752</v>
       </c>
       <c r="CF118" s="6" t="n">
         <v>0</v>
@@ -19409,7 +19343,7 @@
         <v>9</v>
       </c>
       <c r="CO118" s="1" t="n">
-        <v>40635892.6447752</v>
+        <v>0</v>
       </c>
       <c r="CP118" s="1" t="n">
         <v>0</v>
@@ -19510,7 +19444,7 @@
         <v>0</v>
       </c>
       <c r="CE119" s="6" t="n">
-        <v>40635892.6447752</v>
+        <v>0</v>
       </c>
       <c r="CF119" s="6" t="n">
         <v>0</v>
@@ -19540,7 +19474,7 @@
         <v>0</v>
       </c>
       <c r="CQ119" s="1" t="n">
-        <v>0</v>
+        <v>1050886.8</v>
       </c>
       <c r="CR119" s="1" t="n">
         <v>0</v>
@@ -19575,7 +19509,7 @@
         <v>0</v>
       </c>
       <c r="BK120" s="6" t="n">
-        <v>0</v>
+        <v>1253490.86467101</v>
       </c>
       <c r="BL120" s="6" t="n">
         <v>0</v>
@@ -19665,7 +19599,7 @@
         <v>0</v>
       </c>
       <c r="CQ120" s="1" t="n">
-        <v>1050886.8</v>
+        <v>0</v>
       </c>
       <c r="CR120" s="1" t="n">
         <v>0</v>
@@ -19700,7 +19634,7 @@
         <v>0</v>
       </c>
       <c r="BK121" s="6" t="n">
-        <v>1253490.86467101</v>
+        <v>0</v>
       </c>
       <c r="BL121" s="6" t="n">
         <v>0</v>
@@ -19784,7 +19718,7 @@
         <v>12</v>
       </c>
       <c r="CO121" s="1" t="n">
-        <v>0</v>
+        <v>8005505.001336</v>
       </c>
       <c r="CP121" s="1" t="n">
         <v>0</v>
@@ -19885,7 +19819,7 @@
         <v>0</v>
       </c>
       <c r="CE122" s="6" t="n">
-        <v>0</v>
+        <v>8005505.001336</v>
       </c>
       <c r="CF122" s="6" t="n">
         <v>0</v>
@@ -19909,7 +19843,7 @@
         <v>13</v>
       </c>
       <c r="CO122" s="1" t="n">
-        <v>8005505.001336</v>
+        <v>0</v>
       </c>
       <c r="CP122" s="1" t="n">
         <v>0</v>
@@ -20010,7 +19944,7 @@
         <v>0</v>
       </c>
       <c r="CE123" s="6" t="n">
-        <v>8005505.001336</v>
+        <v>0</v>
       </c>
       <c r="CF123" s="6" t="n">
         <v>0</v>
@@ -20034,7 +19968,7 @@
         <v>14</v>
       </c>
       <c r="CO123" s="1" t="n">
-        <v>0</v>
+        <v>40635892.6447752</v>
       </c>
       <c r="CP123" s="1" t="n">
         <v>0</v>
@@ -20135,7 +20069,7 @@
         <v>0</v>
       </c>
       <c r="CE124" s="6" t="n">
-        <v>0</v>
+        <v>45225402.66558</v>
       </c>
       <c r="CF124" s="6" t="n">
         <v>0</v>
@@ -20159,7 +20093,7 @@
         <v>15</v>
       </c>
       <c r="CO124" s="1" t="n">
-        <v>45225402.66558</v>
+        <v>0</v>
       </c>
       <c r="CP124" s="1" t="n">
         <v>0</v>
@@ -20197,7 +20131,7 @@
         <v>0</v>
       </c>
       <c r="BJ125" s="6" t="n">
-        <v>0</v>
+        <v>27853.346068534</v>
       </c>
       <c r="BK125" s="6" t="n">
         <v>0</v>
@@ -20260,7 +20194,7 @@
         <v>0</v>
       </c>
       <c r="CE125" s="6" t="n">
-        <v>45225402.66558</v>
+        <v>0</v>
       </c>
       <c r="CF125" s="6" t="n">
         <v>0</v>
@@ -20322,19 +20256,19 @@
         <v>0</v>
       </c>
       <c r="BJ126" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK126" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL126" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM126" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN126" s="6" t="n">
         <v>27853.346068534</v>
-      </c>
-      <c r="BK126" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL126" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM126" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN126" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="BO126" s="6" t="n">
         <v>0</v>
@@ -20453,13 +20387,13 @@
         <v>0</v>
       </c>
       <c r="BL127" s="6" t="n">
-        <v>0</v>
+        <v>199847.318978253</v>
       </c>
       <c r="BM127" s="6" t="n">
         <v>0</v>
       </c>
       <c r="BN127" s="6" t="n">
-        <v>27853.346068534</v>
+        <v>0</v>
       </c>
       <c r="BO127" s="6" t="n">
         <v>0</v>
@@ -20578,16 +20512,16 @@
         <v>0</v>
       </c>
       <c r="BL128" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM128" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN128" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO128" s="6" t="n">
         <v>199847.318978253</v>
-      </c>
-      <c r="BM128" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN128" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO128" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="BP128" s="6" t="n">
         <v>0</v>
@@ -20712,7 +20646,7 @@
         <v>0</v>
       </c>
       <c r="BO129" s="6" t="n">
-        <v>199847.318978253</v>
+        <v>0</v>
       </c>
       <c r="BP129" s="6" t="n">
         <v>0</v>
@@ -20784,7 +20718,7 @@
         <v>20</v>
       </c>
       <c r="CO129" s="1" t="n">
-        <v>0</v>
+        <v>13528049.1087492</v>
       </c>
       <c r="CP129" s="1" t="n">
         <v>0</v>
@@ -20885,7 +20819,7 @@
         <v>0</v>
       </c>
       <c r="CE130" s="6" t="n">
-        <v>0</v>
+        <v>13528049.1087492</v>
       </c>
       <c r="CF130" s="6" t="n">
         <v>0</v>
@@ -20909,7 +20843,7 @@
         <v>21</v>
       </c>
       <c r="CO130" s="1" t="n">
-        <v>13528049.1087492</v>
+        <v>0</v>
       </c>
       <c r="CP130" s="1" t="n">
         <v>0</v>
@@ -20926,7 +20860,7 @@
         <v>22</v>
       </c>
       <c r="BC131" s="6" t="n">
-        <v>0</v>
+        <v>3347317.4724324</v>
       </c>
       <c r="BD131" s="6" t="n">
         <v>0</v>
@@ -21010,7 +20944,7 @@
         <v>0</v>
       </c>
       <c r="CE131" s="6" t="n">
-        <v>13528049.1087492</v>
+        <v>0</v>
       </c>
       <c r="CF131" s="6" t="n">
         <v>0</v>
@@ -21159,7 +21093,7 @@
         <v>23</v>
       </c>
       <c r="CO132" s="1" t="n">
-        <v>0</v>
+        <v>45225402.66558</v>
       </c>
       <c r="CP132" s="1" t="n">
         <v>0</v>
@@ -21168,7 +21102,7 @@
         <v>0</v>
       </c>
       <c r="CR132" s="1" t="n">
-        <v>3347317.4724324</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
@@ -21176,7 +21110,7 @@
         <v>24</v>
       </c>
       <c r="BC133" s="6" t="n">
-        <v>3347317.4724324</v>
+        <v>0</v>
       </c>
       <c r="BD133" s="6" t="n">
         <v>0</v>
@@ -21293,7 +21227,7 @@
         <v>0</v>
       </c>
       <c r="CR133" s="1" t="n">
-        <v>0</v>
+        <v>1891512.504</v>
       </c>
     </row>
     <row r="134">
@@ -21495,7 +21429,7 @@
         <v>0</v>
       </c>
       <c r="BZ135" s="6" t="n">
-        <v>0</v>
+        <v>1891512.504</v>
       </c>
       <c r="CA135" s="6" t="n">
         <v>0</v>
@@ -21543,7 +21477,7 @@
         <v>0</v>
       </c>
       <c r="CR135" s="1" t="n">
-        <v>1891512.504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -21617,10 +21551,10 @@
         <v>0</v>
       </c>
       <c r="BY136" s="6" t="n">
-        <v>0</v>
+        <v>2521699.4809766</v>
       </c>
       <c r="BZ136" s="6" t="n">
-        <v>1891512.504</v>
+        <v>0</v>
       </c>
       <c r="CA136" s="6" t="n">
         <v>0</v>
@@ -21679,7 +21613,7 @@
         <v>0</v>
       </c>
       <c r="BD137" s="6" t="n">
-        <v>0</v>
+        <v>14862828.8108352</v>
       </c>
       <c r="BE137" s="6" t="n">
         <v>0</v>
@@ -21742,7 +21676,7 @@
         <v>0</v>
       </c>
       <c r="BY137" s="6" t="n">
-        <v>2521699.4809766</v>
+        <v>0</v>
       </c>
       <c r="BZ137" s="6" t="n">
         <v>0</v>
@@ -21804,43 +21738,43 @@
         <v>0</v>
       </c>
       <c r="BD138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO138" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP138" s="6" t="n">
         <v>14862828.8108352</v>
-      </c>
-      <c r="BE138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO138" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP138" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="BQ138" s="6" t="n">
         <v>0</v>
@@ -21965,7 +21899,7 @@
         <v>0</v>
       </c>
       <c r="BP139" s="6" t="n">
-        <v>14862828.8108352</v>
+        <v>0</v>
       </c>
       <c r="BQ139" s="6" t="n">
         <v>0</v>
@@ -22004,7 +21938,7 @@
         <v>0</v>
       </c>
       <c r="CC139" s="6" t="n">
-        <v>0</v>
+        <v>391031.372077766</v>
       </c>
       <c r="CD139" s="6" t="n">
         <v>0</v>
@@ -22093,7 +22027,7 @@
         <v>0</v>
       </c>
       <c r="BQ140" s="6" t="n">
-        <v>0</v>
+        <v>391031.372077766</v>
       </c>
       <c r="BR140" s="6" t="n">
         <v>0</v>
@@ -22129,7 +22063,7 @@
         <v>0</v>
       </c>
       <c r="CC140" s="6" t="n">
-        <v>391031.372077766</v>
+        <v>0</v>
       </c>
       <c r="CD140" s="6" t="n">
         <v>0</v>
@@ -22218,7 +22152,7 @@
         <v>0</v>
       </c>
       <c r="BQ141" s="6" t="n">
-        <v>391031.372077766</v>
+        <v>0</v>
       </c>
       <c r="BR141" s="6" t="n">
         <v>0</v>
@@ -22263,10 +22197,10 @@
         <v>0</v>
       </c>
       <c r="CF141" s="6" t="n">
-        <v>0</v>
+        <v>121834.370880332</v>
       </c>
       <c r="CG141" s="6" t="n">
-        <v>0</v>
+        <v>108477908.839307</v>
       </c>
       <c r="CH141" s="6" t="n">
         <v>0</v>
@@ -22382,16 +22316,16 @@
         <v>0</v>
       </c>
       <c r="CD142" s="6" t="n">
-        <v>0</v>
+        <v>108599743.210187</v>
       </c>
       <c r="CE142" s="6" t="n">
         <v>0</v>
       </c>
       <c r="CF142" s="6" t="n">
-        <v>121834.370880332</v>
+        <v>0</v>
       </c>
       <c r="CG142" s="6" t="n">
-        <v>108477908.839307</v>
+        <v>0</v>
       </c>
       <c r="CH142" s="6" t="n">
         <v>0</v>
@@ -22507,7 +22441,7 @@
         <v>0</v>
       </c>
       <c r="CD143" s="6" t="n">
-        <v>108599743.210187</v>
+        <v>0</v>
       </c>
       <c r="CE143" s="6" t="n">
         <v>0</v>
@@ -22525,7 +22459,7 @@
         <v>0</v>
       </c>
       <c r="CJ143" s="6" t="n">
-        <v>0</v>
+        <v>1763.36022332228</v>
       </c>
       <c r="CK143" s="6" t="n">
         <v>0</v>
@@ -22596,7 +22530,7 @@
         <v>0</v>
       </c>
       <c r="BR144" s="6" t="n">
-        <v>0</v>
+        <v>1763.36022332228</v>
       </c>
       <c r="BS144" s="6" t="n">
         <v>0</v>
@@ -22650,7 +22584,7 @@
         <v>0</v>
       </c>
       <c r="CJ144" s="6" t="n">
-        <v>1763.36022332228</v>
+        <v>0</v>
       </c>
       <c r="CK144" s="6" t="n">
         <v>0</v>
@@ -22721,7 +22655,7 @@
         <v>0</v>
       </c>
       <c r="BR145" s="6" t="n">
-        <v>1763.36022332228</v>
+        <v>0</v>
       </c>
       <c r="BS145" s="6" t="n">
         <v>0</v>
@@ -22793,7 +22727,7 @@
         <v>0</v>
       </c>
       <c r="CR145" s="1" t="n">
-        <v>0</v>
+        <v>3347317.4724324</v>
       </c>
     </row>
     <row r="146">
@@ -24782,46 +24716,46 @@
         <v>0</v>
       </c>
       <c r="X164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ164" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK164" s="6" t="n">
         <v>3347317.4724324</v>
-      </c>
-      <c r="Y164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ164" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK164" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="AL164" s="6" t="n">
         <v>0</v>
@@ -24934,13 +24868,13 @@
         <v>0</v>
       </c>
       <c r="W165" s="6" t="n">
-        <v>0</v>
+        <v>3347317.4724324</v>
       </c>
       <c r="X165" s="6" t="n">
         <v>0</v>
       </c>
       <c r="Y165" s="6" t="n">
-        <v>3347317.4724324</v>
+        <v>0</v>
       </c>
       <c r="Z165" s="6" t="n">
         <v>0</v>
@@ -25056,10 +24990,10 @@
         <v>0</v>
       </c>
       <c r="L166" s="6" t="n">
-        <v>0</v>
+        <v>29154.7439580188</v>
       </c>
       <c r="M166" s="6" t="n">
-        <v>29154.7439580188</v>
+        <v>0</v>
       </c>
       <c r="N166" s="6" t="n">
         <v>0</v>
@@ -25193,10 +25127,10 @@
         <v>0</v>
       </c>
       <c r="F167" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G167" s="6" t="n">
         <v>5353.1838648</v>
-      </c>
-      <c r="G167" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="H167" s="6" t="n">
         <v>0</v>
@@ -25342,7 +25276,7 @@
         <v>0</v>
       </c>
       <c r="D168" s="6" t="n">
-        <v>0</v>
+        <v>5353.1838648</v>
       </c>
       <c r="E168" s="6" t="n">
         <v>0</v>
@@ -25351,7 +25285,7 @@
         <v>0</v>
       </c>
       <c r="G168" s="6" t="n">
-        <v>5353.1838648</v>
+        <v>0</v>
       </c>
       <c r="H168" s="6" t="n">
         <v>0</v>
@@ -25497,10 +25431,10 @@
         <v>0</v>
       </c>
       <c r="D169" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E169" s="6" t="n">
         <v>1230889.29702133</v>
-      </c>
-      <c r="E169" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="F169" s="6" t="n">
         <v>0</v>
@@ -25676,10 +25610,10 @@
         <v>0</v>
       </c>
       <c r="L170" s="6" t="n">
-        <v>0</v>
+        <v>482347.932595389</v>
       </c>
       <c r="M170" s="6" t="n">
-        <v>482347.932595389</v>
+        <v>0</v>
       </c>
       <c r="N170" s="6" t="n">
         <v>0</v>
@@ -25831,10 +25765,10 @@
         <v>0</v>
       </c>
       <c r="L171" s="6" t="n">
-        <v>0</v>
+        <v>4178.0019102801</v>
       </c>
       <c r="M171" s="6" t="n">
-        <v>4178.0019102801</v>
+        <v>0</v>
       </c>
       <c r="N171" s="6" t="n">
         <v>0</v>
@@ -25983,10 +25917,10 @@
         <v>0</v>
       </c>
       <c r="K172" s="6" t="n">
-        <v>0</v>
+        <v>1050886.8</v>
       </c>
       <c r="L172" s="6" t="n">
-        <v>1050886.8</v>
+        <v>0</v>
       </c>
       <c r="M172" s="6" t="n">
         <v>0</v>
@@ -26141,10 +26075,10 @@
         <v>0</v>
       </c>
       <c r="L173" s="6" t="n">
-        <v>0</v>
+        <v>199847.318978253</v>
       </c>
       <c r="M173" s="6" t="n">
-        <v>199847.318978253</v>
+        <v>0</v>
       </c>
       <c r="N173" s="6" t="n">
         <v>0</v>
@@ -26466,10 +26400,10 @@
         <v>0</v>
       </c>
       <c r="Q175" s="6" t="n">
-        <v>0</v>
+        <v>27853.346068534</v>
       </c>
       <c r="R175" s="6" t="n">
-        <v>27853.346068534</v>
+        <v>0</v>
       </c>
       <c r="S175" s="6" t="n">
         <v>0</v>
@@ -26627,10 +26561,10 @@
         <v>0</v>
       </c>
       <c r="S176" s="6" t="n">
-        <v>0</v>
+        <v>199847.318978253</v>
       </c>
       <c r="T176" s="6" t="n">
-        <v>199847.318978253</v>
+        <v>0</v>
       </c>
       <c r="U176" s="6" t="n">
         <v>0</v>
@@ -26812,10 +26746,10 @@
         <v>0</v>
       </c>
       <c r="AC177" s="6" t="n">
-        <v>0</v>
+        <v>14862828.8108352</v>
       </c>
       <c r="AD177" s="6" t="n">
-        <v>14862828.8108352</v>
+        <v>0</v>
       </c>
       <c r="AE177" s="6" t="n">
         <v>0</v>
@@ -26973,10 +26907,10 @@
         <v>0</v>
       </c>
       <c r="AE178" s="6" t="n">
-        <v>0</v>
+        <v>391031.372077766</v>
       </c>
       <c r="AF178" s="6" t="n">
-        <v>391031.372077766</v>
+        <v>0</v>
       </c>
       <c r="AG178" s="6" t="n">
         <v>0</v>
@@ -27140,10 +27074,10 @@
         <v>0</v>
       </c>
       <c r="AI179" s="6" t="n">
-        <v>0</v>
+        <v>1763.36022332228</v>
       </c>
       <c r="AJ179" s="6" t="n">
-        <v>1763.36022332228</v>
+        <v>0</v>
       </c>
       <c r="AK179" s="6" t="n">
         <v>0</v>
@@ -28350,13 +28284,13 @@
         <v>0</v>
       </c>
       <c r="Y187" s="6" t="n">
-        <v>0</v>
+        <v>1891512.504</v>
       </c>
       <c r="Z187" s="6" t="n">
         <v>0</v>
       </c>
       <c r="AA187" s="6" t="n">
-        <v>1891512.504</v>
+        <v>0</v>
       </c>
       <c r="AB187" s="6" t="n">
         <v>0</v>
@@ -28466,10 +28400,10 @@
         <v>0</v>
       </c>
       <c r="L188" s="6" t="n">
-        <v>0</v>
+        <v>287979.207184906</v>
       </c>
       <c r="M188" s="6" t="n">
-        <v>287979.207184906</v>
+        <v>0</v>
       </c>
       <c r="N188" s="6" t="n">
         <v>0</v>
@@ -28666,10 +28600,10 @@
         <v>0</v>
       </c>
       <c r="AA189" s="6" t="n">
-        <v>0</v>
+        <v>1891512.504</v>
       </c>
       <c r="AB189" s="6" t="n">
-        <v>1891512.504</v>
+        <v>0</v>
       </c>
       <c r="AC189" s="6" t="n">
         <v>0</v>
@@ -28776,10 +28710,10 @@
         <v>0</v>
       </c>
       <c r="L190" s="6" t="n">
-        <v>0</v>
+        <v>129040.352785663</v>
       </c>
       <c r="M190" s="6" t="n">
-        <v>129040.352785663</v>
+        <v>0</v>
       </c>
       <c r="N190" s="6" t="n">
         <v>0</v>
@@ -28994,10 +28928,10 @@
         <v>0</v>
       </c>
       <c r="AG191" s="6" t="n">
-        <v>0</v>
+        <v>108599743.210187</v>
       </c>
       <c r="AH191" s="6" t="n">
-        <v>108599743.210187</v>
+        <v>0</v>
       </c>
       <c r="AI191" s="6" t="n">
         <v>0</v>
@@ -29080,49 +29014,49 @@
         <v>0</v>
       </c>
       <c r="J192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M192" s="6" t="n">
+        <v>8005505.001336</v>
+      </c>
+      <c r="N192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O192" s="6" t="n">
         <v>40635892.6447752</v>
       </c>
-      <c r="K192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N192" s="6" t="n">
-        <v>8005505.001336</v>
-      </c>
-      <c r="O192" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="P192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U192" s="6" t="n">
+        <v>13528049.1087492</v>
+      </c>
+      <c r="V192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W192" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X192" s="6" t="n">
         <v>45225402.66558</v>
-      </c>
-      <c r="Q192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V192" s="6" t="n">
-        <v>13528049.1087492</v>
-      </c>
-      <c r="W192" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X192" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="Y192" s="6" t="n">
         <v>0</v>
@@ -29241,10 +29175,10 @@
         <v>0</v>
       </c>
       <c r="L193" s="6" t="n">
-        <v>0</v>
+        <v>41699.5746616493</v>
       </c>
       <c r="M193" s="6" t="n">
-        <v>41699.5746616493</v>
+        <v>0</v>
       </c>
       <c r="N193" s="6" t="n">
         <v>0</v>
@@ -29390,10 +29324,10 @@
         <v>0</v>
       </c>
       <c r="J194" s="6" t="n">
-        <v>0</v>
+        <v>40635892.6447752</v>
       </c>
       <c r="K194" s="6" t="n">
-        <v>40635892.6447752</v>
+        <v>0</v>
       </c>
       <c r="L194" s="6" t="n">
         <v>0</v>
@@ -29402,16 +29336,16 @@
         <v>0</v>
       </c>
       <c r="N194" s="6" t="n">
-        <v>0</v>
+        <v>8005505.001336</v>
       </c>
       <c r="O194" s="6" t="n">
-        <v>8005505.001336</v>
+        <v>0</v>
       </c>
       <c r="P194" s="6" t="n">
-        <v>0</v>
+        <v>45225402.66558</v>
       </c>
       <c r="Q194" s="6" t="n">
-        <v>45225402.66558</v>
+        <v>0</v>
       </c>
       <c r="R194" s="6" t="n">
         <v>0</v>
@@ -29426,10 +29360,10 @@
         <v>0</v>
       </c>
       <c r="V194" s="6" t="n">
-        <v>0</v>
+        <v>13528049.1087492</v>
       </c>
       <c r="W194" s="6" t="n">
-        <v>13528049.1087492</v>
+        <v>0</v>
       </c>
       <c r="X194" s="6" t="n">
         <v>0</v>
@@ -29551,10 +29485,10 @@
         <v>0</v>
       </c>
       <c r="L195" s="6" t="n">
-        <v>0</v>
+        <v>21713.0770261717</v>
       </c>
       <c r="M195" s="6" t="n">
-        <v>21713.0770261717</v>
+        <v>0</v>
       </c>
       <c r="N195" s="6" t="n">
         <v>0</v>
@@ -29706,10 +29640,10 @@
         <v>0</v>
       </c>
       <c r="L196" s="6" t="n">
-        <v>0</v>
+        <v>531.037727366206</v>
       </c>
       <c r="M196" s="6" t="n">
-        <v>531.037727366206</v>
+        <v>0</v>
       </c>
       <c r="N196" s="6" t="n">
         <v>0</v>
@@ -29861,10 +29795,10 @@
         <v>0</v>
       </c>
       <c r="L197" s="6" t="n">
-        <v>0</v>
+        <v>1814.46941507861</v>
       </c>
       <c r="M197" s="6" t="n">
-        <v>1814.46941507861</v>
+        <v>0</v>
       </c>
       <c r="N197" s="6" t="n">
         <v>0</v>
@@ -30016,10 +29950,10 @@
         <v>0</v>
       </c>
       <c r="L198" s="6" t="n">
-        <v>0</v>
+        <v>55185.1484282345</v>
       </c>
       <c r="M198" s="6" t="n">
-        <v>55185.1484282345</v>
+        <v>0</v>
       </c>
       <c r="N198" s="6" t="n">
         <v>0</v>
@@ -30311,10 +30245,10 @@
         <v>0</v>
       </c>
       <c r="E203" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F203" s="1" t="n">
         <v>1230889.29702133</v>
-      </c>
-      <c r="F203" s="1" t="n">
-        <v>0</v>
       </c>
       <c r="G203" s="1" t="n">
         <v>0</v>
@@ -30660,10 +30594,10 @@
         <v>0</v>
       </c>
       <c r="R205" s="1" t="n">
-        <v>0</v>
+        <v>27853.346068534</v>
       </c>
       <c r="S205" s="1" t="n">
-        <v>27853.346068534</v>
+        <v>0</v>
       </c>
       <c r="T205" s="1" t="n">
         <v>0</v>
@@ -30821,10 +30755,10 @@
         <v>0</v>
       </c>
       <c r="T206" s="1" t="n">
-        <v>0</v>
+        <v>199847.318978253</v>
       </c>
       <c r="U206" s="1" t="n">
-        <v>199847.318978253</v>
+        <v>0</v>
       </c>
       <c r="V206" s="1" t="n">
         <v>0</v>
@@ -31000,10 +30934,10 @@
         <v>0</v>
       </c>
       <c r="AB207" s="1" t="n">
-        <v>0</v>
+        <v>2521699.4809766</v>
       </c>
       <c r="AC207" s="1" t="n">
-        <v>2521699.4809766</v>
+        <v>0</v>
       </c>
       <c r="AD207" s="1" t="n">
         <v>0</v>
@@ -31161,10 +31095,10 @@
         <v>0</v>
       </c>
       <c r="AD208" s="1" t="n">
-        <v>0</v>
+        <v>14862828.8108352</v>
       </c>
       <c r="AE208" s="1" t="n">
-        <v>14862828.8108352</v>
+        <v>0</v>
       </c>
       <c r="AF208" s="1" t="n">
         <v>0</v>
@@ -31322,10 +31256,10 @@
         <v>0</v>
       </c>
       <c r="AF209" s="1" t="n">
-        <v>0</v>
+        <v>391031.372077766</v>
       </c>
       <c r="AG209" s="1" t="n">
-        <v>391031.372077766</v>
+        <v>0</v>
       </c>
       <c r="AH209" s="1" t="n">
         <v>0</v>
@@ -31483,10 +31417,10 @@
         <v>0</v>
       </c>
       <c r="AH210" s="1" t="n">
-        <v>0</v>
+        <v>108599743.210187</v>
       </c>
       <c r="AI210" s="1" t="n">
-        <v>108599743.210187</v>
+        <v>0</v>
       </c>
       <c r="AJ210" s="1" t="n">
         <v>0</v>
@@ -31644,10 +31578,10 @@
         <v>0</v>
       </c>
       <c r="AJ211" s="1" t="n">
-        <v>0</v>
+        <v>1763.36022332228</v>
       </c>
       <c r="AK211" s="1" t="n">
-        <v>1763.36022332228</v>
+        <v>0</v>
       </c>
       <c r="AL211" s="1" t="n">
         <v>0</v>
@@ -32744,22 +32678,22 @@
         <v>0</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>139</v>
+        <v>72</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="AO1" s="2" t="s">
         <v>77</v>
@@ -32798,49 +32732,49 @@
         <v>89</v>
       </c>
       <c r="BA1" s="2" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="BB1" s="2" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="BC1" s="2" t="s">
         <v>94</v>
       </c>
       <c r="BD1" s="2" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="BE1" s="2" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="BF1" s="2" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="BG1" s="2" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="BH1" s="2" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="BK1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="BL1" s="2" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="BM1" s="2" t="s">
-        <v>139</v>
+        <v>72</v>
       </c>
       <c r="BN1" s="2" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="BO1" s="2" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="BP1" s="2" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="BQ1" s="2" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="BR1" s="2" t="s">
         <v>77</v>
@@ -32879,39 +32813,39 @@
         <v>89</v>
       </c>
       <c r="CD1" s="2" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="CE1" s="2" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="CF1" s="2" t="s">
         <v>94</v>
       </c>
       <c r="CG1" s="2" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="CH1" s="2" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="CI1" s="2" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="CJ1" s="2" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="CK1" s="2" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH2" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AI2" s="7" t="n">
         <v>0</v>
@@ -32992,7 +32926,7 @@
         <v>0</v>
       </c>
       <c r="BK2" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BL2" s="7" t="n">
         <v>0</v>
@@ -33075,13 +33009,13 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AI3" s="7" t="n">
         <v>0</v>
@@ -33162,7 +33096,7 @@
         <v>0</v>
       </c>
       <c r="BK3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BL3" s="7" t="n">
         <v>0</v>
@@ -33245,13 +33179,13 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH4" s="4" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="AI4" s="7" t="n">
         <v>0</v>
@@ -33332,7 +33266,7 @@
         <v>0</v>
       </c>
       <c r="BK4" s="4" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="BL4" s="7" t="n">
         <v>0</v>
@@ -33585,13 +33519,13 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH6" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AI6" s="7" t="n">
         <v>0</v>
@@ -33672,7 +33606,7 @@
         <v>0</v>
       </c>
       <c r="BK6" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BL6" s="7" t="n">
         <v>0</v>
@@ -33755,13 +33689,13 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH7" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AI7" s="7" t="n">
         <v>0</v>
@@ -33842,7 +33776,7 @@
         <v>0</v>
       </c>
       <c r="BK7" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="BL7" s="7" t="n">
         <v>0</v>
@@ -33925,13 +33859,13 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH8" s="4" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="AI8" s="7" t="n">
         <v>0</v>
@@ -34012,7 +33946,7 @@
         <v>0</v>
       </c>
       <c r="BK8" s="4" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="BL8" s="7" t="n">
         <v>0</v>
@@ -34095,13 +34029,13 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH9" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AI9" s="7" t="n">
         <v>0</v>
@@ -34182,7 +34116,7 @@
         <v>0</v>
       </c>
       <c r="BK9" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="BL9" s="7" t="n">
         <v>0</v>
@@ -34265,13 +34199,13 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH10" s="4" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="AI10" s="7" t="n">
         <v>0</v>
@@ -34352,7 +34286,7 @@
         <v>0</v>
       </c>
       <c r="BK10" s="4" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="BL10" s="7" t="n">
         <v>0</v>
@@ -34435,13 +34369,13 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>159</v>
+        <v>138</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH11" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AI11" s="7" t="n">
         <v>0</v>
@@ -34522,7 +34456,7 @@
         <v>0</v>
       </c>
       <c r="BK11" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="BL11" s="7" t="n">
         <v>0</v>
@@ -34605,7 +34539,7 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -34775,13 +34709,13 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH13" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AI13" s="7" t="n">
         <v>0</v>
@@ -34862,7 +34796,7 @@
         <v>0</v>
       </c>
       <c r="BK13" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="BL13" s="7" t="n">
         <v>0</v>
@@ -34945,13 +34879,13 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH14" s="4" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="AI14" s="7" t="n">
         <v>0</v>
@@ -35032,7 +34966,7 @@
         <v>0</v>
       </c>
       <c r="BK14" s="4" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="BL14" s="7" t="n">
         <v>0</v>
@@ -35115,13 +35049,13 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>161</v>
+        <v>140</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH15" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AI15" s="7" t="n">
         <v>0</v>
@@ -35202,7 +35136,7 @@
         <v>0</v>
       </c>
       <c r="BK15" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="BL15" s="7" t="n">
         <v>0</v>
@@ -35285,13 +35219,13 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
       <c r="B16" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH16" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AI16" s="7" t="n">
         <v>0</v>
@@ -35372,7 +35306,7 @@
         <v>0</v>
       </c>
       <c r="BK16" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="BL16" s="7" t="n">
         <v>0</v>
@@ -35455,13 +35389,13 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
       <c r="B17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH17" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AI17" s="7" t="n">
         <v>0</v>
@@ -35542,7 +35476,7 @@
         <v>0</v>
       </c>
       <c r="BK17" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="BL17" s="7" t="n">
         <v>0</v>
@@ -35625,13 +35559,13 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="B18" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH18" s="4" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="AI18" s="7" t="n">
         <v>0</v>
@@ -35712,7 +35646,7 @@
         <v>0</v>
       </c>
       <c r="BK18" s="4" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="BL18" s="7" t="n">
         <v>0</v>
@@ -35795,13 +35729,13 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>165</v>
+        <v>144</v>
       </c>
       <c r="B19" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH19" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AI19" s="7" t="n">
         <v>0</v>
@@ -35882,7 +35816,7 @@
         <v>0</v>
       </c>
       <c r="BK19" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="BL19" s="7" t="n">
         <v>0</v>
@@ -35965,13 +35899,13 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>166</v>
+        <v>145</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH20" s="4" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="AI20" s="7" t="n">
         <v>0</v>
@@ -36052,7 +35986,7 @@
         <v>0</v>
       </c>
       <c r="BK20" s="4" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="BL20" s="7" t="n">
         <v>0</v>
@@ -36135,7 +36069,7 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="s">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>1</v>
@@ -36305,13 +36239,13 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="s">
-        <v>168</v>
+        <v>147</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="AH22" s="4" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="AI22" s="7" t="n">
         <v>0</v>
@@ -36392,7 +36326,7 @@
         <v>0</v>
       </c>
       <c r="BK22" s="4" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="BL22" s="7" t="n">
         <v>0</v>
@@ -36475,7 +36409,7 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>1</v>
@@ -36651,7 +36585,7 @@
         <v>2</v>
       </c>
       <c r="AH24" s="4" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="AI24" s="7" t="n">
         <v>0</v>
@@ -36732,7 +36666,7 @@
         <v>0</v>
       </c>
       <c r="BK24" s="4" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="BL24" s="7" t="n">
         <v>0</v>
@@ -36815,7 +36749,7 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>2</v>
@@ -36985,13 +36919,13 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH26" s="4" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="AI26" s="7" t="n">
         <v>0</v>
@@ -37072,7 +37006,7 @@
         <v>0</v>
       </c>
       <c r="BK26" s="4" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="BL26" s="7" t="n">
         <v>0</v>
@@ -37155,7 +37089,7 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" s="7" t="n">
         <v>2</v>
@@ -37325,13 +37259,13 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B28" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH28" s="4" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="AI28" s="7" t="n">
         <v>0</v>
@@ -37412,7 +37346,7 @@
         <v>0</v>
       </c>
       <c r="BK28" s="4" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="BL28" s="7" t="n">
         <v>0</v>
@@ -37495,7 +37429,7 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B29" s="7" t="n">
         <v>2</v>
@@ -37665,13 +37599,13 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="B30" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH30" s="4" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="AI30" s="7" t="n">
         <v>0</v>
@@ -37752,7 +37686,7 @@
         <v>0</v>
       </c>
       <c r="BK30" s="4" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="BL30" s="7" t="n">
         <v>0</v>
@@ -37835,7 +37769,7 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B31" s="7" t="n">
         <v>2</v>
@@ -38005,7 +37939,7 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="B32" s="7" t="n">
         <v>2</v>
@@ -38029,7 +37963,7 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="s">
-        <v>170</v>
+        <v>118</v>
       </c>
       <c r="B34" s="7" t="n">
         <v>1</v>
@@ -38037,7 +37971,7 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="B35" s="7" t="n">
         <v>2</v>
@@ -38046,22 +37980,22 @@
         <v>0</v>
       </c>
       <c r="AI35" s="2" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="AJ35" s="2" t="s">
-        <v>139</v>
+        <v>72</v>
       </c>
       <c r="AK35" s="2" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="AL35" s="2" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="AM35" s="2" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="AN35" s="2" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="AO35" s="2" t="s">
         <v>77</v>
@@ -38100,28 +38034,28 @@
         <v>89</v>
       </c>
       <c r="BA35" s="2" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="BB35" s="2" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="BC35" s="2" t="s">
         <v>94</v>
       </c>
       <c r="BD35" s="2" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="BE35" s="2" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="BF35" s="2" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="BG35" s="2" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="BH35" s="2" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36">
@@ -38132,7 +38066,7 @@
         <v>2</v>
       </c>
       <c r="AH36" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AI36" s="7" t="n">
         <v>0</v>
@@ -38215,13 +38149,13 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="B37" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH37" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AI37" s="7" t="n">
         <v>0</v>
@@ -38310,7 +38244,7 @@
         <v>2</v>
       </c>
       <c r="AH38" s="4" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="AI38" s="7" t="n">
         <v>6828695.75399502</v>
@@ -38393,7 +38327,7 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="B39" s="7" t="n">
         <v>2</v>
@@ -38488,7 +38422,7 @@
         <v>2</v>
       </c>
       <c r="AH40" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AI40" s="7" t="n">
         <v>0</v>
@@ -38571,13 +38505,13 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="B41" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH41" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AI41" s="7" t="n">
         <v>0</v>
@@ -38666,7 +38600,7 @@
         <v>2</v>
       </c>
       <c r="AH42" s="4" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="AI42" s="7" t="n">
         <v>0</v>
@@ -38749,13 +38683,13 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>2</v>
       </c>
       <c r="AH43" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AI43" s="7" t="n">
         <v>0</v>
@@ -38844,7 +38778,7 @@
         <v>2</v>
       </c>
       <c r="AH44" s="4" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="AI44" s="7" t="n">
         <v>0</v>
@@ -38931,7 +38865,7 @@
         <v>125</v>
       </c>
       <c r="AH45" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AI45" s="7" t="n">
         <v>0</v>
@@ -39097,7 +39031,7 @@
     </row>
     <row r="47">
       <c r="AH47" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AI47" s="7" t="n">
         <v>0</v>
@@ -39180,7 +39114,7 @@
     </row>
     <row r="48">
       <c r="AH48" s="4" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="AI48" s="7" t="n">
         <v>0</v>
@@ -39263,7 +39197,7 @@
     </row>
     <row r="49">
       <c r="AH49" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AI49" s="7" t="n">
         <v>0</v>
@@ -39346,7 +39280,7 @@
     </row>
     <row r="50">
       <c r="AH50" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AI50" s="7" t="n">
         <v>0</v>
@@ -39429,7 +39363,7 @@
     </row>
     <row r="51">
       <c r="AH51" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AI51" s="7" t="n">
         <v>0</v>
@@ -39512,7 +39446,7 @@
     </row>
     <row r="52">
       <c r="AH52" s="4" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="AI52" s="7" t="n">
         <v>0</v>
@@ -39595,7 +39529,7 @@
     </row>
     <row r="53">
       <c r="AH53" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AI53" s="7" t="n">
         <v>0</v>
@@ -39678,7 +39612,7 @@
     </row>
     <row r="54">
       <c r="AH54" s="4" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="AI54" s="7" t="n">
         <v>58916.3269426858</v>
@@ -39844,7 +39778,7 @@
     </row>
     <row r="56">
       <c r="AH56" s="4" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="AI56" s="7" t="n">
         <v>0</v>
@@ -40010,7 +39944,7 @@
     </row>
     <row r="58">
       <c r="AH58" s="4" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="AI58" s="7" t="n">
         <v>0</v>
@@ -40176,7 +40110,7 @@
     </row>
     <row r="60">
       <c r="AH60" s="4" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="AI60" s="7" t="n">
         <v>0</v>
@@ -40342,7 +40276,7 @@
     </row>
     <row r="62">
       <c r="AH62" s="4" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="AI62" s="7" t="n">
         <v>1020812.84580181</v>
@@ -40508,7 +40442,7 @@
     </row>
     <row r="64">
       <c r="AH64" s="4" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="AI64" s="7" t="n">
         <v>0</v>
@@ -40683,22 +40617,22 @@
         <v>0</v>
       </c>
       <c r="AI69" s="2" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="AJ69" s="2" t="s">
-        <v>139</v>
+        <v>72</v>
       </c>
       <c r="AK69" s="2" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="AL69" s="2" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="AM69" s="2" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="AN69" s="2" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="AO69" s="2" t="s">
         <v>77</v>
@@ -40737,52 +40671,52 @@
         <v>89</v>
       </c>
       <c r="BA69" s="2" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="BB69" s="2" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="BC69" s="2" t="s">
         <v>94</v>
       </c>
       <c r="BD69" s="2" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="BE69" s="2" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="BF69" s="2" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="BG69" s="2" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="BH69" s="2" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="BK69" s="3" t="s">
         <v>0</v>
       </c>
       <c r="BL69" s="2" t="s">
-        <v>151</v>
+        <v>130</v>
       </c>
       <c r="BM69" s="2" t="s">
-        <v>152</v>
+        <v>131</v>
       </c>
       <c r="BN69" s="2" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="BO69" s="2" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="BP69" s="2" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="BQ69" s="2" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="BR69" s="2" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="BS69" s="2" t="s">
         <v>106</v>
@@ -40790,7 +40724,7 @@
     </row>
     <row r="70">
       <c r="AH70" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AI70" s="6" t="n">
         <v>0</v>
@@ -40871,7 +40805,7 @@
         <v>0</v>
       </c>
       <c r="BK70" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BL70" s="1" t="n">
         <v>0</v>
@@ -40900,7 +40834,7 @@
     </row>
     <row r="71">
       <c r="AH71" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AI71" s="6" t="n">
         <v>0</v>
@@ -40981,7 +40915,7 @@
         <v>0</v>
       </c>
       <c r="BK71" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BL71" s="1" t="n">
         <v>0</v>
@@ -41010,7 +40944,7 @@
     </row>
     <row r="72">
       <c r="AH72" s="4" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="AI72" s="6" t="n">
         <v>6828695.75399502</v>
@@ -41091,7 +41025,7 @@
         <v>0</v>
       </c>
       <c r="BK72" s="4" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="BL72" s="1" t="n">
         <v>0</v>
@@ -41230,7 +41164,7 @@
     </row>
     <row r="74">
       <c r="AH74" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AI74" s="6" t="n">
         <v>0</v>
@@ -41311,7 +41245,7 @@
         <v>0</v>
       </c>
       <c r="BK74" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BL74" s="1" t="n">
         <v>2310296.3324532</v>
@@ -41340,7 +41274,7 @@
     </row>
     <row r="75">
       <c r="AH75" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AI75" s="6" t="n">
         <v>0</v>
@@ -41421,7 +41355,7 @@
         <v>0</v>
       </c>
       <c r="BK75" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="BL75" s="1" t="n">
         <v>0</v>
@@ -41450,7 +41384,7 @@
     </row>
     <row r="76">
       <c r="AH76" s="4" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="AI76" s="6" t="n">
         <v>0</v>
@@ -41531,7 +41465,7 @@
         <v>0</v>
       </c>
       <c r="BK76" s="4" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="BL76" s="1" t="n">
         <v>0</v>
@@ -41560,7 +41494,7 @@
     </row>
     <row r="77">
       <c r="AH77" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AI77" s="6" t="n">
         <v>0</v>
@@ -41641,7 +41575,7 @@
         <v>0</v>
       </c>
       <c r="BK77" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="BL77" s="1" t="n">
         <v>0</v>
@@ -41670,7 +41604,7 @@
     </row>
     <row r="78">
       <c r="AH78" s="4" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="AI78" s="6" t="n">
         <v>0</v>
@@ -41751,7 +41685,7 @@
         <v>0</v>
       </c>
       <c r="BK78" s="4" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="BL78" s="1" t="n">
         <v>0</v>
@@ -41780,7 +41714,7 @@
     </row>
     <row r="79">
       <c r="AH79" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AI79" s="6" t="n">
         <v>0</v>
@@ -41861,7 +41795,7 @@
         <v>0</v>
       </c>
       <c r="BK79" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="BL79" s="1" t="n">
         <v>0</v>
@@ -42000,7 +41934,7 @@
     </row>
     <row r="81">
       <c r="AH81" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AI81" s="6" t="n">
         <v>0</v>
@@ -42081,7 +42015,7 @@
         <v>0</v>
       </c>
       <c r="BK81" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="BL81" s="1" t="n">
         <v>0</v>
@@ -42110,7 +42044,7 @@
     </row>
     <row r="82">
       <c r="AH82" s="4" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="AI82" s="6" t="n">
         <v>0</v>
@@ -42191,7 +42125,7 @@
         <v>0</v>
       </c>
       <c r="BK82" s="4" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="BL82" s="1" t="n">
         <v>0</v>
@@ -42220,7 +42154,7 @@
     </row>
     <row r="83">
       <c r="AH83" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AI83" s="6" t="n">
         <v>0</v>
@@ -42301,7 +42235,7 @@
         <v>0</v>
       </c>
       <c r="BK83" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="BL83" s="1" t="n">
         <v>0</v>
@@ -42330,7 +42264,7 @@
     </row>
     <row r="84">
       <c r="AH84" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AI84" s="6" t="n">
         <v>0</v>
@@ -42411,7 +42345,7 @@
         <v>0</v>
       </c>
       <c r="BK84" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="BL84" s="1" t="n">
         <v>0</v>
@@ -42440,7 +42374,7 @@
     </row>
     <row r="85">
       <c r="AH85" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AI85" s="6" t="n">
         <v>0</v>
@@ -42521,7 +42455,7 @@
         <v>0</v>
       </c>
       <c r="BK85" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="BL85" s="1" t="n">
         <v>0</v>
@@ -42550,7 +42484,7 @@
     </row>
     <row r="86">
       <c r="AH86" s="4" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="AI86" s="6" t="n">
         <v>0</v>
@@ -42631,7 +42565,7 @@
         <v>0</v>
       </c>
       <c r="BK86" s="4" t="s">
-        <v>131</v>
+        <v>34</v>
       </c>
       <c r="BL86" s="1" t="n">
         <v>0</v>
@@ -42660,7 +42594,7 @@
     </row>
     <row r="87">
       <c r="AH87" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AI87" s="6" t="n">
         <v>0</v>
@@ -42741,7 +42675,7 @@
         <v>0</v>
       </c>
       <c r="BK87" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="BL87" s="1" t="n">
         <v>0</v>
@@ -42770,7 +42704,7 @@
     </row>
     <row r="88">
       <c r="AH88" s="4" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="AI88" s="6" t="n">
         <v>58916.3269426858</v>
@@ -42851,7 +42785,7 @@
         <v>0</v>
       </c>
       <c r="BK88" s="4" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="BL88" s="1" t="n">
         <v>0</v>
@@ -42990,7 +42924,7 @@
     </row>
     <row r="90">
       <c r="AH90" s="4" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="AI90" s="6" t="n">
         <v>0</v>
@@ -43071,7 +43005,7 @@
         <v>0</v>
       </c>
       <c r="BK90" s="4" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="BL90" s="1" t="n">
         <v>0</v>
@@ -43210,7 +43144,7 @@
     </row>
     <row r="92">
       <c r="AH92" s="4" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="AI92" s="6" t="n">
         <v>0</v>
@@ -43291,7 +43225,7 @@
         <v>0</v>
       </c>
       <c r="BK92" s="4" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="BL92" s="1" t="n">
         <v>0</v>
@@ -43430,7 +43364,7 @@
     </row>
     <row r="94">
       <c r="AH94" s="4" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="AI94" s="6" t="n">
         <v>0</v>
@@ -43511,7 +43445,7 @@
         <v>0</v>
       </c>
       <c r="BK94" s="4" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="BL94" s="1" t="n">
         <v>0</v>
@@ -43650,7 +43584,7 @@
     </row>
     <row r="96">
       <c r="AH96" s="4" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="AI96" s="6" t="n">
         <v>1020812.84580181</v>
@@ -43731,7 +43665,7 @@
         <v>0</v>
       </c>
       <c r="BK96" s="4" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="BL96" s="1" t="n">
         <v>0</v>
@@ -43870,7 +43804,7 @@
     </row>
     <row r="98">
       <c r="AH98" s="4" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="AI98" s="6" t="n">
         <v>0</v>
@@ -43951,7 +43885,7 @@
         <v>4058349.9768</v>
       </c>
       <c r="BK98" s="4" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="BL98" s="1" t="n">
         <v>0</v>
@@ -44103,91 +44037,91 @@
         <v>0</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H103" s="2" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="I103" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J103" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J103" s="2" t="s">
-        <v>129</v>
-      </c>
       <c r="K103" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L103" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M103" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N103" s="2" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="O103" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P103" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="P103" s="2" t="s">
+      <c r="Q103" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="Q103" s="2" t="s">
+      <c r="R103" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="R103" s="2" t="s">
-        <v>131</v>
-      </c>
       <c r="S103" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T103" s="2" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="U103" s="2" t="s">
         <v>40</v>
       </c>
       <c r="V103" s="2" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="W103" s="2" t="s">
         <v>42</v>
       </c>
       <c r="X103" s="2" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="Y103" s="2" t="s">
         <v>44</v>
       </c>
       <c r="Z103" s="2" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="AA103" s="2" t="s">
         <v>46</v>
       </c>
       <c r="AB103" s="2" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="AC103" s="2" t="s">
         <v>48</v>
       </c>
       <c r="AD103" s="2" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="AE103" s="2" t="s">
         <v>50</v>
@@ -44195,7 +44129,7 @@
     </row>
     <row r="104">
       <c r="A104" s="4" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="B104" s="6" t="n">
         <v>0</v>
@@ -44290,7 +44224,7 @@
     </row>
     <row r="105">
       <c r="A105" s="4" t="s">
-        <v>139</v>
+        <v>72</v>
       </c>
       <c r="B105" s="6" t="n">
         <v>95534285.4724076</v>
@@ -44385,7 +44319,7 @@
     </row>
     <row r="106">
       <c r="A106" s="4" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="B106" s="6" t="n">
         <v>0</v>
@@ -44480,7 +44414,7 @@
     </row>
     <row r="107">
       <c r="A107" s="4" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="B107" s="6" t="n">
         <v>0</v>
@@ -44575,7 +44509,7 @@
     </row>
     <row r="108">
       <c r="A108" s="4" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="B108" s="6" t="n">
         <v>0</v>
@@ -44670,7 +44604,7 @@
     </row>
     <row r="109">
       <c r="A109" s="4" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="B109" s="6" t="n">
         <v>0</v>
@@ -45905,7 +45839,7 @@
     </row>
     <row r="122">
       <c r="A122" s="4" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
       <c r="B122" s="6" t="n">
         <v>0</v>
@@ -46000,7 +45934,7 @@
     </row>
     <row r="123">
       <c r="A123" s="4" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="B123" s="6" t="n">
         <v>0</v>
@@ -46190,7 +46124,7 @@
     </row>
     <row r="125">
       <c r="A125" s="4" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="B125" s="6" t="n">
         <v>0</v>
@@ -46285,7 +46219,7 @@
     </row>
     <row r="126">
       <c r="A126" s="4" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="B126" s="6" t="n">
         <v>0</v>
@@ -46380,7 +46314,7 @@
     </row>
     <row r="127">
       <c r="A127" s="4" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="B127" s="6" t="n">
         <v>0</v>
@@ -46475,7 +46409,7 @@
     </row>
     <row r="128">
       <c r="A128" s="4" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="B128" s="6" t="n">
         <v>0</v>
@@ -46570,7 +46504,7 @@
     </row>
     <row r="129">
       <c r="A129" s="4" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="B129" s="6" t="n">
         <v>0</v>
@@ -46674,91 +46608,91 @@
         <v>0</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>126</v>
+        <v>7</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G133" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="I133" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J133" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J133" s="2" t="s">
-        <v>129</v>
-      </c>
       <c r="K133" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L133" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M133" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N133" s="2" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="O133" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P133" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="P133" s="2" t="s">
+      <c r="Q133" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="Q133" s="2" t="s">
+      <c r="R133" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="R133" s="2" t="s">
-        <v>131</v>
-      </c>
       <c r="S133" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T133" s="2" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="U133" s="2" t="s">
         <v>40</v>
       </c>
       <c r="V133" s="2" t="s">
-        <v>133</v>
+        <v>41</v>
       </c>
       <c r="W133" s="2" t="s">
         <v>42</v>
       </c>
       <c r="X133" s="2" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="Y133" s="2" t="s">
         <v>44</v>
       </c>
       <c r="Z133" s="2" t="s">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="AA133" s="2" t="s">
         <v>46</v>
       </c>
       <c r="AB133" s="2" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="AC133" s="2" t="s">
         <v>48</v>
       </c>
       <c r="AD133" s="2" t="s">
-        <v>137</v>
+        <v>49</v>
       </c>
       <c r="AE133" s="2" t="s">
         <v>50</v>

</xml_diff>